<commit_message>
✨ feat: finished xansha templates
</commit_message>
<xml_diff>
--- a/apps/excel-service/templates/XANSHA/Cash Receipt Order.xlsx
+++ b/apps/excel-service/templates/XANSHA/Cash Receipt Order.xlsx
@@ -134,26 +134,26 @@
     <t xml:space="preserve"> Четырнадцать тысячи  восемьсот  тенге 00 тиын</t>
   </si>
   <si>
-    <t>0243</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ринг Ю.А.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Филиал Акционерного общества «Национальная компания «Қазақстан темір жолы» - «Центр диагностики пути» Юр.адрес: 010000, г. Астана, ул. Кунаева, 6, район Есиль, ул. Д. Кунаева, д. 6                Факт.Адрес: г. Астана, ст. Сороковая, ул. Ж. Жабаева, д. 52/2
+    <t>{enumeration}</t>
+  </si>
+  <si>
+    <t>{customer.fullnameClient}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{organization.organization}, {organization.address}
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Основание: Договор                №0243               от  08.06.2026г </t>
+    <t xml:space="preserve">Основание: Договор                №{enumeration}               от  {documentDate.0}г </t>
   </si>
   <si>
     <t xml:space="preserve">за проживание: с 08.06.2026г - 09.06.2026г</t>
   </si>
   <si>
-    <t xml:space="preserve">  20 000  тенге  00 тиын</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Двадцать тысяч тенге 00 тиын</t>
+    <t xml:space="preserve">  {totalPrice}  тенге  00 тиын</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{totalPriceWords} тенге 00 тиын</t>
   </si>
 </sst>
 </file>
@@ -228,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -304,6 +304,15 @@
     </xf>
     <xf fontId="4" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="2" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1911,7 +1920,7 @@
       </c>
       <c r="D127" s="11"/>
       <c r="E127" s="11"/>
-      <c r="F127" s="5" t="s">
+      <c r="F127" s="26" t="s">
         <v>39</v>
       </c>
       <c r="G127" s="5"/>
@@ -1919,7 +1928,7 @@
     </row>
     <row r="128">
       <c r="B128" s="2"/>
-      <c r="C128" s="11" t="s">
+      <c r="C128" s="27" t="s">
         <v>40</v>
       </c>
       <c r="D128" s="11"/>
@@ -1951,7 +1960,7 @@
     </row>
     <row r="131" ht="63" customHeight="1">
       <c r="B131" s="2"/>
-      <c r="C131" s="15" t="s">
+      <c r="C131" s="28" t="s">
         <v>41</v>
       </c>
       <c r="D131" s="15"/>
@@ -1998,7 +2007,7 @@
       <c r="C136" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D136" s="5" t="s">
+      <c r="D136" s="26" t="s">
         <v>43</v>
       </c>
       <c r="E136" s="5"/>
@@ -2008,7 +2017,7 @@
     </row>
     <row r="137">
       <c r="B137" s="2"/>
-      <c r="C137" s="11" t="s">
+      <c r="C137" s="27" t="s">
         <v>44</v>
       </c>
       <c r="D137" s="11"/>

</xml_diff>